<commit_message>
Integrated training data Now, training data on InitialPopulations and EUROMODoutput for PL will be available on GitHub - the user now can run the model immediately using this trating data for PL; Adpated Integartion test to work on both actual and training data - by default it uses training data; to change it to actual data - set `training_flag` to true in `test_run.yml` Also, finalised SimPathsEU_Variable_Codebook
</commit_message>
<xml_diff>
--- a/documentation/SimPathsEU_Schedule.xlsx
+++ b/documentation/SimPathsEU_Schedule.xlsx
@@ -1,28 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pineapple/IdeaProjects/SimPathsEU_APR/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A95EDF4-1240-CD4C-B551-24F3290F091A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D11E36FA-AAEF-D440-AC1F-CBF7337658D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3420" yWindow="2200" windowWidth="42340" windowHeight="23260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="4" r:id="rId1"/>
-    <sheet name="Info fertility" sheetId="3" r:id="rId2"/>
-    <sheet name="Schedule IO disabled" sheetId="1" r:id="rId3"/>
+    <sheet name="Schedule IO disabled" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="172">
   <si>
     <t>Status</t>
   </si>
@@ -457,54 +456,6 @@
     <t>Detail</t>
   </si>
   <si>
-    <t>Why row 21 changed</t>
-  </si>
-  <si>
-    <t>FertilityAlignment uses Parameters.getFertilityRateByYear(year), not projections_fertility.xlsx directly.</t>
-  </si>
-  <si>
-    <t>Runtime target source</t>
-  </si>
-  <si>
-    <t>Parameters.getFertilityRateByYear(year) reads fertilityRateByYear. fertilityRateByYear is built in calculateFertilityRatesFromProjections() from population projections by age/sex/region.</t>
-  </si>
-  <si>
-    <t>Workbook file now shown for row 21</t>
-  </si>
-  <si>
-    <t>align_popProjections.xlsx / Population_projections</t>
-  </si>
-  <si>
-    <t>Where projections_fertility.xlsx is loaded</t>
-  </si>
-  <si>
-    <t>Parameters.loadParameters() loads projections_fertility.xlsx sheet FertilityByYear into fertilityProjectionsByYear.</t>
-  </si>
-  <si>
-    <t>Where projections_fertility.xlsx is used in runtime code</t>
-  </si>
-  <si>
-    <t>Person regressor source FertilityRate uses Parameters.getFertilityProjectionsByYear(year) only when ioFlag=true.</t>
-  </si>
-  <si>
-    <t>Normal simulation path</t>
-  </si>
-  <si>
-    <t>When ioFlag=false, Person regressor source FertilityRate uses Parameters.getFertilityRateByRegionYear(region, year), which is also derived from population projections.</t>
-  </si>
-  <si>
-    <t>Other uses</t>
-  </si>
-  <si>
-    <t>Parameters.getFertilityProjectionsByYear(...) is also used in parameter/time-series support code and bounds handling, but not as the direct FertilityAlignment target.</t>
-  </si>
-  <si>
-    <t>Key code paths</t>
-  </si>
-  <si>
-    <t>FertilityAlignment.java line 32; Parameters.java lines 1420-1449, 1153, 3018-3022; Person.java lines 2849-2853.</t>
-  </si>
-  <si>
     <t>SimPathsEU Schedule Notes</t>
   </si>
   <si>
@@ -614,21 +565,6 @@
   </si>
   <si>
     <t>Outcome-variable descriptions are high-value summaries. Some methods update additional helper fields, temporary state, or linked objects.</t>
-  </si>
-  <si>
-    <t>Related sheets</t>
-  </si>
-  <si>
-    <t>Info</t>
-  </si>
-  <si>
-    <t>Short note explaining the meaning of the start-year column.</t>
-  </si>
-  <si>
-    <t>Info fertility</t>
-  </si>
-  <si>
-    <t>Specific note on why FertilityAlignment is documented against population projections rather than projections_fertility.xlsx as the direct runtime target source.</t>
   </si>
   <si>
     <t>The sheet "Schedule IO disabled" represents the yearly schedule built in SimPathsModel.buildSchedule() for the standard SimPaths configuration with enableIntertemporalOptimisations=false.</t>
@@ -638,7 +574,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -675,11 +611,6 @@
     </font>
     <font>
       <b/>
-      <sz val="12"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <b/>
       <sz val="14"/>
       <name val="Aptos Narrow"/>
     </font>
@@ -694,18 +625,12 @@
       <name val="Aptos Narrow"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -943,24 +868,50 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
@@ -969,69 +920,59 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1039,44 +980,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1411,7 +1321,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1419,218 +1329,200 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="20">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="17">
+      <c r="A3" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="17">
+      <c r="A4" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B4" s="6"/>
+    </row>
+    <row r="5" spans="1:2" ht="34">
+      <c r="A5" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="34">
+      <c r="A6" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="34">
+      <c r="A7" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="17">
+      <c r="A8" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="B8" s="6"/>
+    </row>
+    <row r="9" spans="1:2" ht="17">
+      <c r="A9" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="17">
+      <c r="A10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="17">
+      <c r="A11" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="17">
+      <c r="A12" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="34">
+      <c r="A13" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="17">
+      <c r="A14" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="B1" s="66" t="s">
+    </row>
+    <row r="15" spans="1:2" ht="34">
+      <c r="A15" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="17">
-      <c r="A3" s="67" t="s">
-        <v>132</v>
-      </c>
-      <c r="B3" s="67" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="17">
-      <c r="A4" s="68" t="s">
+    <row r="16" spans="1:2" ht="17">
+      <c r="A16" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="B4" s="69"/>
-    </row>
-    <row r="5" spans="1:2" ht="34">
-      <c r="A5" s="70" t="s">
+    </row>
+    <row r="17" spans="1:2" ht="17">
+      <c r="A17" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="B5" s="70" t="s">
+      <c r="B17" s="6"/>
+    </row>
+    <row r="18" spans="1:2" ht="34">
+      <c r="A18" s="7" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="34">
-      <c r="A6" s="70" t="s">
+      <c r="B18" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="B6" s="70" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="34">
-      <c r="A7" s="70" t="s">
+    </row>
+    <row r="19" spans="1:2" ht="34">
+      <c r="A19" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="B7" s="70" t="s">
+      <c r="B19" s="7" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="17">
-      <c r="A8" s="68" t="s">
+    <row r="20" spans="1:2" ht="17">
+      <c r="A20" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="B8" s="69"/>
-    </row>
-    <row r="9" spans="1:2" ht="17">
-      <c r="A9" s="70" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="70" t="s">
+      <c r="B20" s="7" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="17">
-      <c r="A10" s="70" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="70" t="s">
+    <row r="21" spans="1:2" ht="17">
+      <c r="A21" s="7" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" ht="17">
-      <c r="A11" s="70" t="s">
+      <c r="B21" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="B11" s="70" t="s">
+    </row>
+    <row r="22" spans="1:2" ht="17">
+      <c r="A22" s="7" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" ht="17">
-      <c r="A12" s="70" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" s="70" t="s">
+      <c r="B22" s="7" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="34">
-      <c r="A13" s="70" t="s">
+    <row r="23" spans="1:2" ht="34">
+      <c r="A23" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="B13" s="70" t="s">
+      <c r="B23" s="6"/>
+    </row>
+    <row r="24" spans="1:2" ht="34">
+      <c r="A24" s="7" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" ht="17">
-      <c r="A14" s="70" t="s">
-        <v>7</v>
-      </c>
-      <c r="B14" s="70" t="s">
+      <c r="B24" s="7" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="34">
-      <c r="A15" s="70" t="s">
-        <v>8</v>
-      </c>
-      <c r="B15" s="70" t="s">
+    <row r="25" spans="1:2" ht="34">
+      <c r="A25" s="7" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" ht="17">
-      <c r="A16" s="70" t="s">
-        <v>9</v>
-      </c>
-      <c r="B16" s="70" t="s">
+      <c r="B25" s="7" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17">
-      <c r="A17" s="68" t="s">
+    <row r="26" spans="1:2" ht="17">
+      <c r="A26" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="B17" s="69"/>
-    </row>
-    <row r="18" spans="1:2" ht="34">
-      <c r="A18" s="70" t="s">
+      <c r="B26" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="B18" s="70" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="34">
-      <c r="A19" s="70" t="s">
-        <v>172</v>
-      </c>
-      <c r="B19" s="70" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="17">
-      <c r="A20" s="70" t="s">
-        <v>174</v>
-      </c>
-      <c r="B20" s="70" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="17">
-      <c r="A21" s="70" t="s">
-        <v>176</v>
-      </c>
-      <c r="B21" s="70" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="17">
-      <c r="A22" s="70" t="s">
-        <v>178</v>
-      </c>
-      <c r="B22" s="70" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="34">
-      <c r="A23" s="68" t="s">
-        <v>180</v>
-      </c>
-      <c r="B23" s="69"/>
-    </row>
-    <row r="24" spans="1:2" ht="34">
-      <c r="A24" s="70" t="s">
-        <v>181</v>
-      </c>
-      <c r="B24" s="70" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="34">
-      <c r="A25" s="70" t="s">
-        <v>183</v>
-      </c>
-      <c r="B25" s="70" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="17">
-      <c r="A26" s="70" t="s">
-        <v>185</v>
-      </c>
-      <c r="B26" s="70" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="17">
-      <c r="A27" s="68" t="s">
-        <v>187</v>
-      </c>
-      <c r="B27" s="69"/>
-    </row>
-    <row r="28" spans="1:2" ht="17">
-      <c r="A28" s="70" t="s">
-        <v>188</v>
-      </c>
-      <c r="B28" s="70" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="34">
-      <c r="A29" s="70" t="s">
-        <v>190</v>
-      </c>
-      <c r="B29" s="70" t="s">
-        <v>191</v>
-      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="7"/>
+      <c r="B27" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1638,98 +1530,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
-  <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="120" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" ht="17" customHeight="1">
-      <c r="A1" s="63" t="s">
-        <v>132</v>
-      </c>
-      <c r="B1" s="63" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="17" customHeight="1">
-      <c r="A2" s="64" t="s">
-        <v>134</v>
-      </c>
-      <c r="B2" s="64" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="34" customHeight="1">
-      <c r="A3" s="64" t="s">
-        <v>136</v>
-      </c>
-      <c r="B3" s="64" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="34" customHeight="1">
-      <c r="A4" s="64" t="s">
-        <v>138</v>
-      </c>
-      <c r="B4" s="64" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="34" customHeight="1">
-      <c r="A5" s="64" t="s">
-        <v>140</v>
-      </c>
-      <c r="B5" s="64" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="34" customHeight="1">
-      <c r="A6" s="64" t="s">
-        <v>142</v>
-      </c>
-      <c r="B6" s="64" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="34" customHeight="1">
-      <c r="A7" s="64" t="s">
-        <v>144</v>
-      </c>
-      <c r="B7" s="64" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="34" customHeight="1">
-      <c r="A8" s="64" t="s">
-        <v>146</v>
-      </c>
-      <c r="B8" s="64" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="17" customHeight="1">
-      <c r="A9" s="64" t="s">
-        <v>148</v>
-      </c>
-      <c r="B9" s="64" t="s">
-        <v>149</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="9.6640625" customWidth="1"/>
-    <col min="2" max="2" width="8" style="12" customWidth="1"/>
+    <col min="2" max="2" width="8" style="1" customWidth="1"/>
     <col min="3" max="3" width="27.83203125" customWidth="1"/>
     <col min="4" max="4" width="8" customWidth="1"/>
     <col min="5" max="5" width="50.1640625" customWidth="1"/>
@@ -1742,952 +1548,952 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35" customHeight="1" thickBot="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="57" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="22" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="23" t="s">
+      <c r="E1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="25" t="s">
+      <c r="G1" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="26" t="s">
+      <c r="I1" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="26" t="s">
+      <c r="J1" s="15" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="17" customHeight="1">
-      <c r="A2" s="28"/>
-      <c r="B2" s="58">
+      <c r="A2" s="16"/>
+      <c r="B2" s="17">
         <v>1</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="17"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="18" t="s">
+      <c r="G2" s="21"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="J2" s="18"/>
+      <c r="J2" s="22"/>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="29"/>
-      <c r="B3" s="39">
+      <c r="A3" s="23"/>
+      <c r="B3" s="24">
         <v>2</v>
       </c>
       <c r="C3" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="25" t="s">
         <v>11</v>
       </c>
       <c r="E3" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="6"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="1" t="s">
+      <c r="G3" s="26"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J3" s="1"/>
+      <c r="J3" s="27"/>
     </row>
     <row r="4" spans="1:10" ht="17" customHeight="1">
-      <c r="A4" s="29"/>
-      <c r="B4" s="39">
+      <c r="A4" s="23"/>
+      <c r="B4" s="24">
         <v>3</v>
       </c>
       <c r="C4" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="6"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="1" t="s">
+      <c r="G4" s="26"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="1"/>
+      <c r="J4" s="27"/>
     </row>
     <row r="5" spans="1:10" ht="102" customHeight="1">
-      <c r="A5" s="44"/>
-      <c r="B5" s="39">
+      <c r="A5" s="29"/>
+      <c r="B5" s="24">
         <v>4</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="35" t="s">
+      <c r="E5" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="8"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="37" t="s">
+      <c r="G5" s="32"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="37"/>
+      <c r="J5" s="33"/>
     </row>
     <row r="6" spans="1:10" ht="104" customHeight="1" thickBot="1">
-      <c r="A6" s="45"/>
-      <c r="B6" s="59">
+      <c r="A6" s="34"/>
+      <c r="B6" s="35">
         <v>5</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="46" t="s">
+      <c r="E6" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="11"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="47" t="s">
+      <c r="G6" s="39"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="J6" s="47"/>
+      <c r="J6" s="40"/>
     </row>
     <row r="7" spans="1:10" ht="17" customHeight="1">
-      <c r="A7" s="28"/>
-      <c r="B7" s="58">
+      <c r="A7" s="16"/>
+      <c r="B7" s="17">
         <v>6</v>
       </c>
-      <c r="C7" s="36" t="s">
+      <c r="C7" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="32" t="s">
+      <c r="D7" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="24" t="s">
+      <c r="E7" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="32" t="s">
+      <c r="F7" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="G7" s="33" t="s">
+      <c r="G7" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="H7" s="32" t="s">
+      <c r="H7" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="I7" s="18" t="s">
+      <c r="I7" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="J7" s="18"/>
+      <c r="J7" s="22"/>
     </row>
     <row r="8" spans="1:10" ht="34" customHeight="1">
-      <c r="A8" s="31" t="s">
+      <c r="A8" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="38">
+      <c r="B8" s="24">
         <v>7</v>
       </c>
-      <c r="C8" s="40" t="s">
+      <c r="C8" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="40" t="s">
+      <c r="D8" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="41" t="s">
+      <c r="E8" s="45" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="40" t="s">
+      <c r="F8" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="41" t="s">
+      <c r="G8" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="H8" s="41" t="s">
+      <c r="H8" s="45" t="s">
         <v>34</v>
       </c>
-      <c r="I8" s="19" t="s">
+      <c r="I8" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="J8" s="19"/>
+      <c r="J8" s="27"/>
     </row>
     <row r="9" spans="1:10" ht="17" customHeight="1">
-      <c r="A9" s="29"/>
-      <c r="B9" s="39">
+      <c r="A9" s="23"/>
+      <c r="B9" s="24">
         <v>8</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="44" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="34" t="s">
+      <c r="E9" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="44" t="s">
         <v>38</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="H9" s="44" t="s">
         <v>39</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="I9" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J9" s="1"/>
+      <c r="J9" s="27"/>
     </row>
     <row r="10" spans="1:10" ht="51" customHeight="1">
-      <c r="A10" s="29"/>
-      <c r="B10" s="39">
+      <c r="A10" s="23"/>
+      <c r="B10" s="24">
         <v>9</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="44" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="34" t="s">
+      <c r="E10" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="44" t="s">
         <v>42</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="44" t="s">
         <v>43</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="I10" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J10" s="1"/>
+      <c r="J10" s="27"/>
     </row>
     <row r="11" spans="1:10" ht="34" customHeight="1">
-      <c r="A11" s="60"/>
-      <c r="B11" s="39">
+      <c r="A11" s="46"/>
+      <c r="B11" s="24">
         <v>10</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="E11" s="34" t="s">
+      <c r="E11" s="45" t="s">
         <v>45</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="34" t="s">
+      <c r="G11" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="H11" s="51" t="s">
+      <c r="H11" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="I11" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="J11" s="1"/>
+      <c r="J11" s="27"/>
     </row>
     <row r="12" spans="1:10" ht="51" customHeight="1">
-      <c r="A12" s="29"/>
-      <c r="B12" s="39">
+      <c r="A12" s="23"/>
+      <c r="B12" s="24">
         <v>11</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="E12" s="34" t="s">
+      <c r="E12" s="45" t="s">
         <v>50</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="44" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="H12" s="44" t="s">
         <v>51</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="I12" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J12" s="1"/>
+      <c r="J12" s="27"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="60"/>
-      <c r="B13" s="39">
+      <c r="A13" s="46"/>
+      <c r="B13" s="24">
         <v>12</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="44" t="s">
         <v>52</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4" t="s">
+      <c r="E13" s="44"/>
+      <c r="F13" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="H13" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="I13" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="J13" s="27" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="17" customHeight="1">
-      <c r="A14" s="29"/>
-      <c r="B14" s="39">
+      <c r="A14" s="23"/>
+      <c r="B14" s="24">
         <v>13</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="44" t="s">
         <v>57</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="34" t="s">
+      <c r="E14" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="44" t="s">
         <v>59</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="H14" s="44" t="s">
         <v>60</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="I14" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J14" s="1"/>
+      <c r="J14" s="27"/>
     </row>
     <row r="15" spans="1:10" ht="34" customHeight="1">
-      <c r="A15" s="31" t="s">
+      <c r="A15" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="38">
+      <c r="B15" s="24">
         <v>14</v>
       </c>
-      <c r="C15" s="40" t="s">
+      <c r="C15" s="44" t="s">
         <v>61</v>
       </c>
-      <c r="D15" s="40" t="s">
+      <c r="D15" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="41" t="s">
+      <c r="E15" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="F15" s="40" t="s">
+      <c r="F15" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="G15" s="41" t="s">
+      <c r="G15" s="45" t="s">
         <v>63</v>
       </c>
-      <c r="H15" s="41" t="s">
+      <c r="H15" s="45" t="s">
         <v>64</v>
       </c>
-      <c r="I15" s="19" t="s">
+      <c r="I15" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="J15" s="19"/>
+      <c r="J15" s="27"/>
     </row>
     <row r="16" spans="1:10" ht="17" customHeight="1">
-      <c r="A16" s="29"/>
-      <c r="B16" s="39">
+      <c r="A16" s="23"/>
+      <c r="B16" s="24">
         <v>15</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="44" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="E16" s="34" t="s">
+      <c r="E16" s="45" t="s">
         <v>67</v>
       </c>
-      <c r="F16" s="43" t="s">
+      <c r="F16" s="48" t="s">
         <v>24</v>
       </c>
-      <c r="G16" s="43" t="s">
+      <c r="G16" s="48" t="s">
         <v>68</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="H16" s="44" t="s">
         <v>69</v>
       </c>
-      <c r="I16" s="1" t="s">
+      <c r="I16" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J16" s="1"/>
+      <c r="J16" s="27"/>
     </row>
     <row r="17" spans="1:10" ht="34" customHeight="1">
-      <c r="A17" s="29"/>
-      <c r="B17" s="39">
+      <c r="A17" s="23"/>
+      <c r="B17" s="24">
         <v>16</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="44" t="s">
         <v>70</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="E17" s="34" t="s">
+      <c r="E17" s="45" t="s">
         <v>71</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F17" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="G17" s="34" t="s">
+      <c r="G17" s="45" t="s">
         <v>72</v>
       </c>
-      <c r="H17" s="34" t="s">
+      <c r="H17" s="45" t="s">
         <v>73</v>
       </c>
-      <c r="I17" s="1" t="s">
+      <c r="I17" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J17" s="1"/>
+      <c r="J17" s="27"/>
     </row>
     <row r="18" spans="1:10" ht="34" customHeight="1">
-      <c r="A18" s="60"/>
-      <c r="B18" s="39">
+      <c r="A18" s="46"/>
+      <c r="B18" s="24">
         <v>17</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="44" t="s">
         <v>74</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="E18" s="34" t="s">
+      <c r="E18" s="45" t="s">
         <v>75</v>
       </c>
-      <c r="F18" s="43" t="s">
+      <c r="F18" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="G18" s="62" t="s">
+      <c r="G18" s="49" t="s">
         <v>76</v>
       </c>
-      <c r="H18" s="34" t="s">
+      <c r="H18" s="45" t="s">
         <v>77</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="I18" s="27" t="s">
         <v>78</v>
       </c>
-      <c r="J18" s="1"/>
+      <c r="J18" s="27"/>
     </row>
     <row r="19" spans="1:10" ht="17" customHeight="1">
-      <c r="A19" s="29"/>
-      <c r="B19" s="39">
+      <c r="A19" s="23"/>
+      <c r="B19" s="24">
         <v>18</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="44" t="s">
         <v>79</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="34" t="s">
+      <c r="E19" s="45" t="s">
         <v>80</v>
       </c>
-      <c r="F19" s="43" t="s">
+      <c r="F19" s="48" t="s">
         <v>24</v>
       </c>
-      <c r="G19" s="43" t="s">
+      <c r="G19" s="48" t="s">
         <v>81</v>
       </c>
-      <c r="H19" s="4" t="s">
+      <c r="H19" s="44" t="s">
         <v>82</v>
       </c>
-      <c r="I19" s="1" t="s">
+      <c r="I19" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J19" s="1"/>
+      <c r="J19" s="27"/>
     </row>
     <row r="20" spans="1:10" ht="34" customHeight="1">
-      <c r="A20" s="29"/>
-      <c r="B20" s="39">
+      <c r="A20" s="23"/>
+      <c r="B20" s="24">
         <v>19</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="44" t="s">
         <v>83</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="E20" s="34" t="s">
+      <c r="E20" s="45" t="s">
         <v>84</v>
       </c>
-      <c r="F20" s="43" t="s">
+      <c r="F20" s="48" t="s">
         <v>24</v>
       </c>
-      <c r="G20" s="43"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="1" t="s">
+      <c r="G20" s="48"/>
+      <c r="H20" s="44"/>
+      <c r="I20" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J20" s="1"/>
+      <c r="J20" s="27"/>
     </row>
     <row r="21" spans="1:10" ht="17" customHeight="1">
-      <c r="A21" s="29"/>
-      <c r="B21" s="39">
+      <c r="A21" s="23"/>
+      <c r="B21" s="24">
         <v>20</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="44" t="s">
         <v>85</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="42" t="s">
+      <c r="E21" s="50" t="s">
         <v>86</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="G21" s="44" t="s">
         <v>87</v>
       </c>
-      <c r="H21" s="4" t="s">
+      <c r="H21" s="44" t="s">
         <v>88</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="I21" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J21" s="1"/>
+      <c r="J21" s="27"/>
     </row>
     <row r="22" spans="1:10" ht="37" customHeight="1">
-      <c r="A22" s="29"/>
-      <c r="B22" s="39">
+      <c r="A22" s="23"/>
+      <c r="B22" s="24">
         <v>21</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="44" t="s">
         <v>89</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="E22" s="34" t="s">
+      <c r="E22" s="45" t="s">
         <v>90</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="G22" s="34" t="s">
+      <c r="G22" s="45" t="s">
         <v>91</v>
       </c>
-      <c r="H22" s="34" t="s">
+      <c r="H22" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="I22" s="1" t="s">
+      <c r="I22" s="27" t="s">
         <v>93</v>
       </c>
-      <c r="J22" s="1"/>
+      <c r="J22" s="27"/>
     </row>
     <row r="23" spans="1:10" ht="17" customHeight="1">
-      <c r="A23" s="29"/>
-      <c r="B23" s="39">
+      <c r="A23" s="23"/>
+      <c r="B23" s="24">
         <v>22</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="44" t="s">
         <v>94</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="E23" s="34" t="s">
+      <c r="E23" s="45" t="s">
         <v>95</v>
       </c>
-      <c r="F23" s="43" t="s">
+      <c r="F23" s="48" t="s">
         <v>24</v>
       </c>
-      <c r="G23" s="43" t="s">
+      <c r="G23" s="48" t="s">
         <v>96</v>
       </c>
-      <c r="H23" s="4" t="s">
+      <c r="H23" s="44" t="s">
         <v>97</v>
       </c>
-      <c r="I23" s="1" t="s">
+      <c r="I23" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J23" s="1"/>
+      <c r="J23" s="27"/>
     </row>
     <row r="24" spans="1:10" ht="17" customHeight="1">
-      <c r="A24" s="29"/>
-      <c r="B24" s="39">
+      <c r="A24" s="23"/>
+      <c r="B24" s="24">
         <v>23</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="44" t="s">
         <v>98</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="E24" s="42" t="s">
+      <c r="E24" s="50" t="s">
         <v>99</v>
       </c>
-      <c r="F24" s="43" t="s">
+      <c r="F24" s="48" t="s">
         <v>24</v>
       </c>
-      <c r="G24" s="43"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="37" t="s">
+      <c r="G24" s="48"/>
+      <c r="H24" s="25"/>
+      <c r="I24" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="J24" s="37"/>
+      <c r="J24" s="33"/>
     </row>
     <row r="25" spans="1:10" ht="94" customHeight="1">
-      <c r="A25" s="29"/>
-      <c r="B25" s="39">
+      <c r="A25" s="23"/>
+      <c r="B25" s="24">
         <v>24</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="44" t="s">
         <v>100</v>
       </c>
-      <c r="D25" s="34" t="s">
+      <c r="D25" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="E25" s="34" t="s">
+      <c r="E25" s="45" t="s">
         <v>101</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="F25" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="G25" s="34" t="s">
+      <c r="G25" s="45" t="s">
         <v>102</v>
       </c>
-      <c r="H25" s="34" t="s">
+      <c r="H25" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="I25" s="61" t="s">
+      <c r="I25" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="J25" s="1"/>
+      <c r="J25" s="27"/>
     </row>
     <row r="26" spans="1:10" ht="17" customHeight="1">
-      <c r="A26" s="29"/>
-      <c r="B26" s="39">
+      <c r="A26" s="23"/>
+      <c r="B26" s="24">
         <v>25</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="44" t="s">
         <v>105</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="E26" s="34" t="s">
+      <c r="E26" s="45" t="s">
         <v>106</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="1" t="s">
+      <c r="G26" s="44"/>
+      <c r="H26" s="44"/>
+      <c r="I26" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J26" s="1"/>
+      <c r="J26" s="27"/>
     </row>
     <row r="27" spans="1:10" ht="17" customHeight="1">
-      <c r="A27" s="29"/>
-      <c r="B27" s="39">
+      <c r="A27" s="23"/>
+      <c r="B27" s="24">
         <v>26</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="44" t="s">
         <v>107</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="E27" s="34" t="s">
+      <c r="E27" s="45" t="s">
         <v>108</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F27" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="5" t="s">
+      <c r="G27" s="44"/>
+      <c r="H27" s="44"/>
+      <c r="I27" s="52" t="s">
         <v>14</v>
       </c>
-      <c r="J27" s="5"/>
+      <c r="J27" s="52"/>
     </row>
     <row r="28" spans="1:10" ht="34" customHeight="1">
-      <c r="A28" s="29"/>
-      <c r="B28" s="39">
+      <c r="A28" s="23"/>
+      <c r="B28" s="24">
         <v>27</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="44" t="s">
         <v>109</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="E28" s="34" t="s">
+      <c r="E28" s="45" t="s">
         <v>110</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="G28" s="44" t="s">
         <v>111</v>
       </c>
-      <c r="H28" s="4" t="s">
+      <c r="H28" s="44" t="s">
         <v>112</v>
       </c>
-      <c r="I28" s="5" t="s">
+      <c r="I28" s="52" t="s">
         <v>14</v>
       </c>
-      <c r="J28" s="5"/>
+      <c r="J28" s="52"/>
     </row>
     <row r="29" spans="1:10" ht="15" customHeight="1">
-      <c r="A29" s="29"/>
-      <c r="B29" s="39">
+      <c r="A29" s="23"/>
+      <c r="B29" s="24">
         <v>28</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="44" t="s">
         <v>113</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="E29" s="34" t="s">
+      <c r="E29" s="45" t="s">
         <v>114</v>
       </c>
-      <c r="F29" s="4" t="s">
+      <c r="F29" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="G29" s="34" t="s">
+      <c r="G29" s="45" t="s">
         <v>115</v>
       </c>
-      <c r="H29" s="2"/>
-      <c r="I29" s="1" t="s">
+      <c r="H29" s="25"/>
+      <c r="I29" s="27" t="s">
         <v>116</v>
       </c>
-      <c r="J29" s="1"/>
+      <c r="J29" s="27"/>
     </row>
     <row r="30" spans="1:10" ht="52" customHeight="1" thickBot="1">
-      <c r="A30" s="30"/>
-      <c r="B30" s="59">
+      <c r="A30" s="53"/>
+      <c r="B30" s="35">
         <v>29</v>
       </c>
-      <c r="C30" s="52" t="s">
+      <c r="C30" s="54" t="s">
         <v>117</v>
       </c>
-      <c r="D30" s="53" t="s">
+      <c r="D30" s="55" t="s">
         <v>11</v>
       </c>
-      <c r="E30" s="53"/>
-      <c r="F30" s="53" t="s">
+      <c r="E30" s="55"/>
+      <c r="F30" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="G30" s="54" t="s">
+      <c r="G30" s="56" t="s">
         <v>118</v>
       </c>
-      <c r="H30" s="55"/>
-      <c r="I30" s="56" t="s">
+      <c r="H30" s="57"/>
+      <c r="I30" s="58" t="s">
         <v>119</v>
       </c>
-      <c r="J30" s="56" t="s">
+      <c r="J30" s="58" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="34" customHeight="1">
-      <c r="A31" s="48"/>
-      <c r="B31" s="58">
+      <c r="A31" s="59"/>
+      <c r="B31" s="17">
         <v>30</v>
       </c>
-      <c r="C31" s="49" t="s">
+      <c r="C31" s="60" t="s">
         <v>121</v>
       </c>
-      <c r="D31" s="50" t="s">
+      <c r="D31" s="61" t="s">
         <v>26</v>
       </c>
-      <c r="E31" s="35" t="s">
+      <c r="E31" s="31" t="s">
         <v>122</v>
       </c>
-      <c r="F31" s="50" t="s">
+      <c r="F31" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="G31" s="33"/>
-      <c r="H31" s="32"/>
-      <c r="I31" s="18" t="s">
+      <c r="G31" s="43"/>
+      <c r="H31" s="42"/>
+      <c r="I31" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="J31" s="18"/>
+      <c r="J31" s="22"/>
     </row>
     <row r="32" spans="1:10">
-      <c r="A32" s="29"/>
-      <c r="B32" s="39">
+      <c r="A32" s="23"/>
+      <c r="B32" s="24">
         <v>31</v>
       </c>
-      <c r="C32" s="12" t="s">
+      <c r="C32" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="D32" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="E32" s="12"/>
-      <c r="F32" s="7" t="s">
+      <c r="E32" s="1"/>
+      <c r="F32" s="30" t="s">
         <v>125</v>
       </c>
-      <c r="G32" s="8"/>
-      <c r="H32" s="7"/>
-      <c r="I32" s="1" t="s">
+      <c r="G32" s="32"/>
+      <c r="H32" s="30"/>
+      <c r="I32" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J32" s="1"/>
+      <c r="J32" s="27"/>
     </row>
     <row r="33" spans="1:10">
-      <c r="A33" s="29"/>
-      <c r="B33" s="39">
+      <c r="A33" s="23"/>
+      <c r="B33" s="24">
         <v>32</v>
       </c>
-      <c r="C33" s="12" t="s">
+      <c r="C33" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D33" s="7" t="s">
+      <c r="D33" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="E33" s="12" t="s">
+      <c r="E33" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="F33" s="7" t="s">
+      <c r="F33" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="G33" s="8"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="1" t="s">
+      <c r="G33" s="32"/>
+      <c r="H33" s="30"/>
+      <c r="I33" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J33" s="1"/>
+      <c r="J33" s="27"/>
     </row>
     <row r="34" spans="1:10">
-      <c r="A34" s="29"/>
-      <c r="B34" s="39">
+      <c r="A34" s="23"/>
+      <c r="B34" s="24">
         <v>33</v>
       </c>
-      <c r="C34" s="12" t="s">
+      <c r="C34" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="D34" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="E34" s="12" t="s">
+      <c r="E34" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="F34" s="7" t="s">
+      <c r="F34" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="G34" s="8"/>
-      <c r="H34" s="7"/>
-      <c r="I34" s="1" t="s">
+      <c r="G34" s="32"/>
+      <c r="H34" s="30"/>
+      <c r="I34" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J34" s="1"/>
+      <c r="J34" s="27"/>
     </row>
     <row r="35" spans="1:10">
-      <c r="A35" s="29"/>
-      <c r="B35" s="39">
+      <c r="A35" s="23"/>
+      <c r="B35" s="24">
         <v>34</v>
       </c>
-      <c r="C35" s="12" t="s">
+      <c r="C35" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="D35" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="E35" s="12"/>
-      <c r="F35" s="7" t="s">
+      <c r="E35" s="1"/>
+      <c r="F35" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="G35" s="8"/>
-      <c r="H35" s="7"/>
-      <c r="I35" s="1" t="s">
+      <c r="G35" s="32"/>
+      <c r="H35" s="30"/>
+      <c r="I35" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J35" s="1"/>
+      <c r="J35" s="27"/>
     </row>
     <row r="36" spans="1:10" ht="18" customHeight="1" thickBot="1">
-      <c r="A36" s="30"/>
-      <c r="B36" s="59">
+      <c r="A36" s="53"/>
+      <c r="B36" s="35">
         <v>35</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="C36" s="36" t="s">
         <v>130</v>
       </c>
-      <c r="D36" s="10" t="s">
+      <c r="D36" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="E36" s="20" t="s">
+      <c r="E36" s="62" t="s">
         <v>131</v>
       </c>
-      <c r="F36" s="10" t="s">
+      <c r="F36" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="G36" s="11"/>
-      <c r="H36" s="10"/>
-      <c r="I36" s="3" t="s">
+      <c r="G36" s="39"/>
+      <c r="H36" s="37"/>
+      <c r="I36" s="63" t="s">
         <v>14</v>
       </c>
-      <c r="J36" s="3"/>
+      <c r="J36" s="63"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>